<commit_message>
Updated CTISum excel sheet
</commit_message>
<xml_diff>
--- a/#-CATHARINA_BENCHMARKING_RESULTS/CTISum-Vision_results/CTISum-Vision_results.xlsx
+++ b/#-CATHARINA_BENCHMARKING_RESULTS/CTISum-Vision_results/CTISum-Vision_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studntnu.sharepoint.com/sites/o365_BachelorBoys2026/Shared Documents/General/Test results/CTISum/CTISum_Vision_Results_V2_1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1030" documentId="11_109AA5FC69E05A0FD18DCD9610509E723B73F6F9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B05B54BF-4817-4A75-82C7-9243D7022963}"/>
+  <xr:revisionPtr revIDLastSave="1034" documentId="11_109AA5FC69E05A0FD18DCD9610509E723B73F6F9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3155D9A0-6A35-409E-9CAA-465850D63F59}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -164,7 +164,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -275,11 +275,219 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -327,25 +535,91 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="23" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="26" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -608,7 +882,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{18E5297D-0C6D-4AB4-9D51-C94CC02E2AF9}" type="CELLRANGE">
+                    <a:fld id="{1D192E0D-E285-4CAA-A845-2FED868EF94D}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -641,7 +915,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9D9D72AD-B222-42EC-80A0-8033CB230E89}" type="CELLRANGE">
+                    <a:fld id="{7B105865-E304-45C1-8074-2D8B8E1F5B37}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -675,7 +949,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{492BC764-242C-44B0-ADE1-1B9EB5ED002A}" type="CELLRANGE">
+                    <a:fld id="{EBB6374B-61FE-4597-AA0F-154561B249D5}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -709,7 +983,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{12605986-3D5B-4F79-9882-1AC4D787BB60}" type="CELLRANGE">
+                    <a:fld id="{DECBFEA0-D152-463D-A18B-1C819FC99CAC}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -743,7 +1017,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{107E3CCF-93F4-4ED6-830D-2BF9D49E1A41}" type="CELLRANGE">
+                    <a:fld id="{8C9635FA-6190-437C-B100-910F530B1BF0}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -1445,7 +1719,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6D1333DC-AFE5-40AE-8E71-D5FB04112567}" type="CELLRANGE">
+                    <a:fld id="{0050DCA4-A028-47EC-9978-0B7A66FA94D1}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -1478,7 +1752,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{4F318B14-160C-45E9-A714-6BA1AC872E88}" type="CELLRANGE">
+                    <a:fld id="{AECAE369-0395-4545-A4B0-11B6682DC3F3}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -1518,7 +1792,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A0317CD7-3032-4592-A2E2-865AABBFAE88}" type="CELLRANGE">
+                    <a:fld id="{C27D8F5C-D282-4AEE-A3FC-3FEB9D08D09D}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -1551,7 +1825,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{35E55EB4-44DA-483B-9FAF-9A2D35BE7849}" type="CELLRANGE">
+                    <a:fld id="{99488886-B4B1-46BC-B098-3D54D3634739}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -1585,7 +1859,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9E87EB61-5940-4016-8D24-F07AF78DD666}" type="CELLRANGE">
+                    <a:fld id="{E353090A-6112-4BB5-B099-D5962A9B1254}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -2386,7 +2660,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5576AF57-A9F7-4D85-868A-44A011CEE1AE}" type="CELLRANGE">
+                    <a:fld id="{8D8FDE53-D30E-4594-AFF6-8205F86F8E01}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -2425,7 +2699,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E26AFA47-3AF5-4B47-891E-30F807F0ABAC}" type="CELLRANGE">
+                    <a:fld id="{80E60F81-EED5-4A62-83A1-CD617FDA42A7}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -2478,7 +2752,7 @@
                         <a:cs typeface="+mn-cs"/>
                       </a:defRPr>
                     </a:pPr>
-                    <a:fld id="{CC7633DB-4ED5-4C9F-98E5-B95D52900163}" type="CELLRANGE">
+                    <a:fld id="{51626BF7-C091-4369-A1B8-E48AE2F47E7C}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr>
                         <a:defRPr sz="1200"/>
@@ -2554,7 +2828,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C0F15EB9-0733-4C40-9A66-45B421F8F135}" type="CELLRANGE">
+                    <a:fld id="{DBCB2BA2-8D4E-4F08-99F3-518B48B71906}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -2592,7 +2866,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7935FCB8-4FB7-4D53-B6EB-9F6D6B560166}" type="CELLRANGE">
+                    <a:fld id="{A995A41A-5650-461F-A9C6-EA4311504367}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -3390,7 +3664,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{30CD653F-F828-499B-9B5F-9CDB4BE5182F}" type="CELLRANGE">
+                    <a:fld id="{9746E29D-8766-4016-B26B-937D32F42548}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -3429,7 +3703,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C80C033B-A62F-42AF-8996-25EFFDDE6A42}" type="CELLRANGE">
+                    <a:fld id="{BC57E156-FECF-4D06-BCB0-E47A0228A9DA}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -3468,7 +3742,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D947AF34-7B6F-47D3-A27F-67A3928DCADB}" type="CELLRANGE">
+                    <a:fld id="{0F2DA375-EFD7-45FE-BE41-624AFD9EBC47}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -3507,7 +3781,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B50CC050-6129-4F5A-B280-8EBB701D8DA5}" type="CELLRANGE">
+                    <a:fld id="{7A495446-31ED-447A-8374-73733AC73778}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -3546,7 +3820,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2C04DD40-E315-4A6D-BFA5-754CD0F24682}" type="CELLRANGE">
+                    <a:fld id="{F4522627-5A67-4514-9AE9-FB5651763A69}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -4194,7 +4468,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{217D580C-EE68-4ECE-89F3-75F88D9624F4}" type="CELLRANGE">
+                    <a:fld id="{CA265E70-10F6-4C09-B157-8372100827E4}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -4233,7 +4507,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1C68B88F-9709-4EB1-9E70-87D85A4561AD}" type="CELLRANGE">
+                    <a:fld id="{A0C5F3E2-20DE-42EB-A598-41A95F936DE1}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -4272,7 +4546,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{CD5FA20C-8341-4734-88A4-FEAC9C888B6F}" type="CELLRANGE">
+                    <a:fld id="{7BB5DA6A-7A44-40EE-9D5E-EA92505E6AE9}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -4311,7 +4585,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{760344F0-61E4-4F3B-B22B-39C93E1D332F}" type="CELLRANGE">
+                    <a:fld id="{BE43AA4D-109C-4AC3-98B7-4C5E6A40230A}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -4350,7 +4624,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{659BC859-31EE-443D-86E5-C0F065444CFA}" type="CELLRANGE">
+                    <a:fld id="{7A005D97-5526-45A1-A154-150E349E7B07}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -5098,7 +5372,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B5657C83-5A66-4555-AF76-C3EA162C9795}" type="CELLRANGE">
+                    <a:fld id="{DA498B08-CB41-4E0E-BB1D-0CB6E1961264}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -5137,7 +5411,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{613EF02B-E908-42E7-991E-1BA797B6E793}" type="CELLRANGE">
+                    <a:fld id="{FB9F67DD-5911-4EFF-9C3B-2312F8137F0A}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -5176,7 +5450,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E3DD5BE7-CD05-4BF3-A5B9-5FADFD9DA4C4}" type="CELLRANGE">
+                    <a:fld id="{DAAD1CBB-9C33-47E6-BD30-34DEC2EBA045}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -5215,7 +5489,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7EBA4217-61F1-4B87-A913-1D77E12050F1}" type="CELLRANGE">
+                    <a:fld id="{705A8820-3362-478E-99A4-DCA89299C75E}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -5254,7 +5528,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{19725BBE-87C3-45A9-90EB-CD83625745E3}" type="CELLRANGE">
+                    <a:fld id="{F7D637DC-B034-4BE1-89F8-FB3776A530E4}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -5996,7 +6270,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8417F668-63DD-45F9-AB29-4D3B5E2A0308}" type="CELLRANGE">
+                    <a:fld id="{B66C9411-A3BD-4B99-9EB8-07482EB06E12}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -6035,7 +6309,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F897B5BC-F7DD-40E3-958A-339304DF35B9}" type="CELLRANGE">
+                    <a:fld id="{382D26AB-573C-4D17-9183-2682850A8F35}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -6074,7 +6348,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E5F61FCC-E755-435A-9A70-0150D7D38B3C}" type="CELLRANGE">
+                    <a:fld id="{2CE9AB2C-15A1-4E1D-A80A-1788C1EEBCB7}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -6113,7 +6387,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{4A82877A-6953-4024-B918-675121672268}" type="CELLRANGE">
+                    <a:fld id="{4575504F-5C9F-43EF-B0B4-3F48C61CE417}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -6152,7 +6426,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D01D4A5D-604B-4B15-A722-BF1F1184A4F0}" type="CELLRANGE">
+                    <a:fld id="{D2DB2F6D-E4D0-4986-A88E-8EB9C48D7F32}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -6890,7 +7164,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{4017C15B-861D-483E-B4F8-16289FD732AE}" type="CELLRANGE">
+                    <a:fld id="{A48F6976-94CB-4807-9FF5-529E50025233}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -6929,7 +7203,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{41277F88-9177-4C09-9ADE-15B22CE4C945}" type="CELLRANGE">
+                    <a:fld id="{31F0E50E-257F-4F14-827F-0E8568B567B9}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -6968,7 +7242,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6A87AC53-C5B9-4D6B-82CE-36507086B207}" type="CELLRANGE">
+                    <a:fld id="{C2BCB6C1-9CE6-4738-8740-C13999A7757A}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -7007,7 +7281,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{802D76C7-71ED-4A0D-8057-8A8421C7B039}" type="CELLRANGE">
+                    <a:fld id="{11853E77-D552-482C-B284-0826E064A39B}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -7046,7 +7320,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2129D98C-535B-4F71-BE7F-183BEB4851B0}" type="CELLRANGE">
+                    <a:fld id="{466B3D8E-072C-4196-8E5C-EF8543F9315B}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLEOMRÅDE]</a:t>
@@ -12686,7 +12960,7 @@
   <dimension ref="D4:T32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="41.54296875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.81640625" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="15.6328125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="23.6328125" bestFit="1" customWidth="1"/>
@@ -12781,10 +13055,10 @@
       <c r="R9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="S9" s="5" t="s">
+      <c r="S9" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="T9" s="5" t="s">
+      <c r="T9" s="26" t="s">
         <v>13</v>
       </c>
     </row>
@@ -12831,10 +13105,10 @@
       <c r="R10" s="7">
         <v>0.27110000000000001</v>
       </c>
-      <c r="S10" s="10">
+      <c r="S10" s="24">
         <v>4.4299999999999999E-2</v>
       </c>
-      <c r="T10" s="10">
+      <c r="T10" s="27">
         <v>0.13589999999999999</v>
       </c>
     </row>
@@ -12881,10 +13155,10 @@
       <c r="R11" s="7">
         <v>0.31090000000000001</v>
       </c>
-      <c r="S11" s="10">
+      <c r="S11" s="24">
         <v>6.54E-2</v>
       </c>
-      <c r="T11" s="10">
+      <c r="T11" s="27">
         <v>0.13980000000000001</v>
       </c>
     </row>
@@ -12931,10 +13205,10 @@
       <c r="R12" s="7">
         <v>0.25879999999999997</v>
       </c>
-      <c r="S12" s="10">
+      <c r="S12" s="24">
         <v>3.5499999999999997E-2</v>
       </c>
-      <c r="T12" s="10">
+      <c r="T12" s="27">
         <v>0.125</v>
       </c>
     </row>
@@ -12970,7 +13244,7 @@
         <v>7</v>
       </c>
       <c r="O13" s="6">
-        <v>2020.89</v>
+        <v>1184.0999999999999</v>
       </c>
       <c r="P13" s="14">
         <v>289</v>
@@ -12981,10 +13255,10 @@
       <c r="R13" s="7">
         <v>0.23730000000000001</v>
       </c>
-      <c r="S13" s="10">
+      <c r="S13" s="24">
         <v>2.5600000000000001E-2</v>
       </c>
-      <c r="T13" s="10">
+      <c r="T13" s="27">
         <v>0.1221</v>
       </c>
     </row>
@@ -13031,10 +13305,10 @@
       <c r="R14" s="9">
         <v>0.26879999999999998</v>
       </c>
-      <c r="S14" s="11">
+      <c r="S14" s="25">
         <v>3.2800000000000003E-2</v>
       </c>
-      <c r="T14" s="10">
+      <c r="T14" s="28">
         <v>0.1479</v>
       </c>
     </row>
@@ -13353,189 +13627,189 @@
       <c r="D27" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="G27" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="H27" s="4" t="s">
+      <c r="H27" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="I27" s="19" t="s">
+      <c r="I27" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="J27" s="19" t="s">
+      <c r="J27" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="K27" s="19" t="s">
+      <c r="K27" s="32" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="28" spans="4:16" x14ac:dyDescent="0.35">
-      <c r="D28" s="20" t="s">
+      <c r="D28" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="E28" s="20">
+      <c r="E28" s="33">
         <f>AVERAGE(E10,E19,N10)</f>
         <v>9</v>
       </c>
-      <c r="F28" s="21">
+      <c r="F28" s="34">
         <f>AVERAGE(F10,F19,O10)</f>
         <v>626.23333333333323</v>
       </c>
-      <c r="G28" s="24">
+      <c r="G28" s="35">
         <f>AVERAGE(G10,G19,P10)</f>
         <v>69.486000000000004</v>
       </c>
-      <c r="H28" s="22">
+      <c r="H28" s="36">
         <f>AVERAGE(H10,H19,Q10)</f>
         <v>0.80646666666666667</v>
       </c>
-      <c r="I28" s="25">
+      <c r="I28" s="37">
         <f>AVERAGE(I10,I19,R10)</f>
         <v>0.2723666666666667</v>
       </c>
-      <c r="J28" s="25">
+      <c r="J28" s="37">
         <f>AVERAGE(J10,J19,S10)</f>
         <v>4.6500000000000007E-2</v>
       </c>
-      <c r="K28" s="25">
+      <c r="K28" s="38">
         <f>AVERAGE(K10,K19,T10)</f>
         <v>0.13639999999999999</v>
       </c>
     </row>
     <row r="29" spans="4:16" x14ac:dyDescent="0.35">
-      <c r="D29" s="20" t="s">
+      <c r="D29" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="E29" s="20">
+      <c r="E29" s="39">
         <f t="shared" ref="E29:E32" si="5">AVERAGE(E11,E20,N11)</f>
         <v>9</v>
       </c>
-      <c r="F29" s="21">
+      <c r="F29" s="19">
         <f t="shared" ref="F29:F32" si="6">AVERAGE(F11,F20,O11)</f>
         <v>849.24333333333334</v>
       </c>
-      <c r="G29" s="24">
+      <c r="G29" s="21">
         <f t="shared" ref="G29:G32" si="7">AVERAGE(G11,G20,P11)</f>
         <v>94.425333333333342</v>
       </c>
-      <c r="H29" s="22">
+      <c r="H29" s="20">
         <f t="shared" ref="H29:H32" si="8">AVERAGE(H11,H20,Q11)</f>
         <v>0.81599999999999995</v>
       </c>
-      <c r="I29" s="25">
+      <c r="I29" s="22">
         <f t="shared" ref="I29:I32" si="9">AVERAGE(I11,I20,R11)</f>
         <v>0.29933333333333328</v>
       </c>
-      <c r="J29" s="25">
+      <c r="J29" s="22">
         <f t="shared" ref="J29:J32" si="10">AVERAGE(J11,J20,S11)</f>
         <v>6.1800000000000001E-2</v>
       </c>
-      <c r="K29" s="25">
+      <c r="K29" s="40">
         <f t="shared" ref="K29:K32" si="11">AVERAGE(K11,K20,T11)</f>
         <v>0.13390000000000002</v>
       </c>
     </row>
     <row r="30" spans="4:16" x14ac:dyDescent="0.35">
-      <c r="D30" s="20" t="s">
+      <c r="D30" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="E30" s="20">
+      <c r="E30" s="39">
         <f t="shared" si="5"/>
         <v>9</v>
       </c>
-      <c r="F30" s="21">
+      <c r="F30" s="19">
         <f t="shared" si="6"/>
         <v>676.34999999999991</v>
       </c>
-      <c r="G30" s="24">
+      <c r="G30" s="21">
         <f t="shared" si="7"/>
         <v>75.053666666666672</v>
       </c>
-      <c r="H30" s="22">
+      <c r="H30" s="20">
         <f t="shared" si="8"/>
         <v>0.7969666666666666</v>
       </c>
-      <c r="I30" s="25">
+      <c r="I30" s="22">
         <f t="shared" si="9"/>
         <v>0.26473333333333332</v>
       </c>
-      <c r="J30" s="25">
+      <c r="J30" s="22">
         <f t="shared" si="10"/>
         <v>4.0333333333333332E-2</v>
       </c>
-      <c r="K30" s="25">
+      <c r="K30" s="40">
         <f t="shared" si="11"/>
         <v>0.12966666666666668</v>
       </c>
     </row>
     <row r="31" spans="4:16" x14ac:dyDescent="0.35">
-      <c r="D31" s="20" t="s">
+      <c r="D31" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="E31" s="24">
+      <c r="E31" s="41">
         <f t="shared" si="5"/>
         <v>7.666666666666667</v>
       </c>
-      <c r="F31" s="21">
+      <c r="F31" s="19">
         <f t="shared" si="6"/>
-        <v>2253.3833333333337</v>
-      </c>
-      <c r="G31" s="24">
+        <v>1974.4533333333336</v>
+      </c>
+      <c r="G31" s="21">
         <f t="shared" si="7"/>
         <v>293.34699999999998</v>
       </c>
-      <c r="H31" s="22">
+      <c r="H31" s="20">
         <f t="shared" si="8"/>
         <v>0.79600000000000015</v>
       </c>
-      <c r="I31" s="25">
+      <c r="I31" s="22">
         <f t="shared" si="9"/>
         <v>0.2359</v>
       </c>
-      <c r="J31" s="25">
+      <c r="J31" s="22">
         <f t="shared" si="10"/>
         <v>2.3033333333333333E-2</v>
       </c>
-      <c r="K31" s="25">
+      <c r="K31" s="40">
         <f t="shared" si="11"/>
         <v>0.11813333333333333</v>
       </c>
     </row>
     <row r="32" spans="4:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D32" s="23" t="s">
+      <c r="D32" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="E32" s="24">
+      <c r="E32" s="42">
         <f t="shared" si="5"/>
         <v>6.333333333333333</v>
       </c>
-      <c r="F32" s="21">
+      <c r="F32" s="43">
         <f t="shared" si="6"/>
         <v>2217.61</v>
       </c>
-      <c r="G32" s="24">
+      <c r="G32" s="44">
         <f t="shared" si="7"/>
         <v>347.3123333333333</v>
       </c>
-      <c r="H32" s="22">
+      <c r="H32" s="45">
         <f t="shared" si="8"/>
         <v>0.80700000000000005</v>
       </c>
-      <c r="I32" s="25">
+      <c r="I32" s="46">
         <f t="shared" si="9"/>
         <v>0.27879999999999999</v>
       </c>
-      <c r="J32" s="25">
+      <c r="J32" s="46">
         <f t="shared" si="10"/>
         <v>3.3900000000000007E-2</v>
       </c>
-      <c r="K32" s="25">
+      <c r="K32" s="47">
         <f t="shared" si="11"/>
         <v>0.15036666666666668</v>
       </c>

</xml_diff>